<commit_message>
chore: update daily stock screen report
</commit_message>
<xml_diff>
--- a/reports/holding_plan.xlsx
+++ b/reports/holding_plan.xlsx
@@ -98,7 +98,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-05 18:54:47</t>
+          <t>2026-09-06 13:41:54</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -311,7 +311,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-05 18:54:47</t>
+          <t>2026-09-06 13:41:54</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -398,7 +398,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-05 18:54:47</t>
+          <t>2026-09-06 13:41:54</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -485,7 +485,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-05 18:54:47</t>
+          <t>2026-09-06 13:41:54</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -572,7 +572,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-05 18:54:47</t>
+          <t>2026-09-06 13:41:54</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -659,7 +659,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-05 18:54:47</t>
+          <t>2026-09-06 13:41:54</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1317,12 +1317,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-12 11:24:52</t>
+          <t>2026-08-12 16:02:51</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>14:40</t>
         </is>
       </c>
       <c r="C2">
@@ -1343,12 +1343,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-12 16:02:51</t>
+          <t>2026-08-13 11:28:14</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C3">
@@ -1369,12 +1369,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-13 11:28:14</t>
+          <t>2026-08-13 16:03:54</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>14:40</t>
         </is>
       </c>
       <c r="C4">
@@ -1395,12 +1395,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-13 16:03:54</t>
+          <t>2026-08-14 11:25:25</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C5">
@@ -1421,12 +1421,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-14 11:25:25</t>
+          <t>2026-08-14 16:00:51</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>14:40</t>
         </is>
       </c>
       <c r="C6">
@@ -1447,12 +1447,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-14 16:00:51</t>
+          <t>2026-08-15 10:14:46</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C7">
@@ -1473,12 +1473,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-15 10:14:46</t>
+          <t>2026-08-15 15:15:06</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>14:40</t>
         </is>
       </c>
       <c r="C8">
@@ -1499,12 +1499,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-15 15:15:06</t>
+          <t>2026-08-16 10:22:31</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C9">
@@ -1525,12 +1525,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-16 10:22:31</t>
+          <t>2026-08-16 15:17:09</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>14:40</t>
         </is>
       </c>
       <c r="C10">
@@ -1551,12 +1551,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-16 15:17:09</t>
+          <t>2026-08-17 10:20:53</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C11">
@@ -1577,12 +1577,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-08-17 10:20:53</t>
+          <t>2026-08-17 15:37:43</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>14:40</t>
         </is>
       </c>
       <c r="C12">
@@ -1603,12 +1603,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-17 15:37:43</t>
+          <t>2026-08-18 10:17:04</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C13">
@@ -1629,12 +1629,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-18 10:17:04</t>
+          <t>2026-08-18 15:23:13</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>14:40</t>
         </is>
       </c>
       <c r="C14">
@@ -1655,12 +1655,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-08-18 15:23:13</t>
+          <t>2026-08-19 10:19:57</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C15">
@@ -1681,12 +1681,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-08-19 10:19:57</t>
+          <t>2026-08-19 15:23:59</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>14:40</t>
         </is>
       </c>
       <c r="C16">
@@ -1707,12 +1707,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-08-19 15:23:59</t>
+          <t>2026-08-20 10:18:26</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C17">
@@ -1733,12 +1733,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-08-20 10:18:26</t>
+          <t>2026-08-20 15:25:49</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>14:40</t>
         </is>
       </c>
       <c r="C18">
@@ -1759,12 +1759,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-08-20 15:25:49</t>
+          <t>2026-08-21 10:24:43</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C19">
@@ -1785,12 +1785,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-21 10:24:43</t>
+          <t>2026-08-21 15:27:09</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>14:40</t>
         </is>
       </c>
       <c r="C20">
@@ -1811,12 +1811,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-21 15:27:09</t>
+          <t>2026-08-22 10:17:12</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C21">
@@ -1837,12 +1837,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-22 10:17:12</t>
+          <t>2026-08-22 15:17:41</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>14:40</t>
         </is>
       </c>
       <c r="C22">
@@ -1863,12 +1863,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-22 15:17:41</t>
+          <t>2026-08-23 10:24:35</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C23">
@@ -1889,12 +1889,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-23 10:24:35</t>
+          <t>2026-08-23 15:19:30</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>14:40</t>
         </is>
       </c>
       <c r="C24">
@@ -1915,12 +1915,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-23 15:19:30</t>
+          <t>2026-08-24 10:23:52</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C25">
@@ -1941,12 +1941,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-24 10:23:52</t>
+          <t>2026-08-24 15:43:12</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>14:40</t>
         </is>
       </c>
       <c r="C26">
@@ -1967,12 +1967,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-24 15:43:12</t>
+          <t>2026-08-25 10:19:24</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C27">
@@ -1993,12 +1993,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-25 10:19:24</t>
+          <t>2026-08-25 15:28:43</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>14:40</t>
         </is>
       </c>
       <c r="C28">
@@ -2019,12 +2019,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-25 15:28:43</t>
+          <t>2026-08-26 10:26:03</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C29">
@@ -2045,12 +2045,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-26 10:26:03</t>
+          <t>2026-08-26 15:30:03</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>14:40</t>
         </is>
       </c>
       <c r="C30">
@@ -2071,7 +2071,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-26 15:30:03</t>
+          <t>2026-08-27 19:02:57</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2097,12 +2097,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-27 19:02:57</t>
+          <t>2026-08-28 01:53:35</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C32">
@@ -2123,12 +2123,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-28 01:53:35</t>
+          <t>2026-08-28 20:36:25</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>14:40</t>
         </is>
       </c>
       <c r="C33">
@@ -2149,12 +2149,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-28 20:36:25</t>
+          <t>2026-08-29 02:59:57</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C34">
@@ -2175,12 +2175,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-29 02:59:57</t>
+          <t>2026-08-29 15:44:45</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>14:40</t>
         </is>
       </c>
       <c r="C35">
@@ -2201,7 +2201,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-29 15:44:45</t>
+          <t>2026-08-29 20:49:51</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2227,7 +2227,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-29 20:49:51</t>
+          <t>2026-08-30 14:22:18</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2253,7 +2253,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-30 14:22:18</t>
+          <t>2026-08-30 20:12:52</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2279,7 +2279,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-30 20:12:52</t>
+          <t>2026-08-31 14:49:59</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2305,7 +2305,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-31 14:49:59</t>
+          <t>2026-08-31 22:24:07</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2331,7 +2331,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-31 22:24:07</t>
+          <t>2026-09-01 14:08:54</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2357,7 +2357,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-09-01 14:08:54</t>
+          <t>2026-09-01 19:59:54</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2383,7 +2383,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-09-01 19:59:54</t>
+          <t>2026-09-02 13:34:22</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2409,7 +2409,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-09-02 13:34:22</t>
+          <t>2026-09-02 19:42:51</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2435,7 +2435,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-09-02 19:42:51</t>
+          <t>2026-09-03 13:35:02</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2461,7 +2461,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-09-03 13:35:02</t>
+          <t>2026-09-03 19:42:36</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2487,7 +2487,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-09-03 19:42:36</t>
+          <t>2026-09-04 13:40:22</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2513,7 +2513,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-09-04 13:40:22</t>
+          <t>2026-09-04 19:43:30</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2539,7 +2539,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-09-04 19:43:30</t>
+          <t>2026-09-05 13:27:07</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2565,7 +2565,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-09-05 13:27:07</t>
+          <t>2026-09-05 18:54:47</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2591,7 +2591,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-09-05 18:54:47</t>
+          <t>2026-09-06 13:41:54</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">

</xml_diff>